<commit_message>
Log transit note for Oct 17: Free Zone arrival 19:03, bus departed 19:23
</commit_message>
<xml_diff>
--- a/omar_elnemr_attendance_2026.xlsx
+++ b/omar_elnemr_attendance_2026.xlsx
@@ -44,7 +44,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -67,6 +67,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FCE4D6"/>
         <bgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -96,7 +102,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -126,6 +132,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -499,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -508,8 +523,8 @@
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="75" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="85" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -1194,14 +1209,54 @@
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="11" t="inlineStr">
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>To Be Updated</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F18" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="11" t="inlineStr">
+        <is>
+          <t>En Route / Transit</t>
+        </is>
+      </c>
+      <c r="H18" s="13" t="inlineStr">
+        <is>
+          <t>🚌 Transit: Arrived Free Zone 07:03 PM, company bus departed 07:23 PM. En route to DAM airport (Awaiting official log-in).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="14" t="inlineStr">
         <is>
           <t>Total October 2026 Hours</t>
         </is>
       </c>
-      <c r="F19" s="12">
-        <f>SUM(F2:F17)</f>
+      <c r="F20" s="15">
+        <f>SUM(F2:F18)</f>
         <v/>
       </c>
     </row>
@@ -1225,8 +1280,8 @@
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="75" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="85" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -1592,12 +1647,12 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="inlineStr">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>Total September 2026 Hours</t>
         </is>
       </c>
-      <c r="F11" s="12">
+      <c r="F11" s="15">
         <f>SUM(F2:F9)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Update Oct 17 shift: Logged in at 08:00 AM (Official Duty)
</commit_message>
<xml_diff>
--- a/omar_elnemr_attendance_2026.xlsx
+++ b/omar_elnemr_attendance_2026.xlsx
@@ -1222,7 +1222,7 @@
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
@@ -1240,12 +1240,12 @@
       </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>En Route / Transit</t>
+          <t>Official Duty</t>
         </is>
       </c>
       <c r="H18" s="13" t="inlineStr">
         <is>
-          <t>🚌 Transit: Arrived Free Zone 07:03 PM, company bus departed 07:23 PM. En route to DAM airport (Awaiting official log-in).</t>
+          <t>✈️ Live Airport Ground Station Duty (Logged in 08:00 AM / Awaiting Checkout | Free Zone Bus: Arr 07:03 PM, Dep 07:23 PM)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Complete Oct 17 shift: Logged out at 03:37 PM (7h 37m)
</commit_message>
<xml_diff>
--- a/omar_elnemr_attendance_2026.xlsx
+++ b/omar_elnemr_attendance_2026.xlsx
@@ -44,7 +44,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -67,12 +67,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FCE4D6"/>
         <bgColor rgb="00FCE4D6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
-        <bgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -102,7 +96,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -132,15 +126,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1210,52 +1195,52 @@
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="11" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="B18" s="11" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>Saturday</t>
         </is>
       </c>
-      <c r="C18" s="11" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>08:00 AM</t>
         </is>
       </c>
-      <c r="D18" s="11" t="inlineStr">
-        <is>
-          <t>To Be Updated</t>
-        </is>
-      </c>
-      <c r="E18" s="11" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="F18" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G18" s="11" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>03:37 PM</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>7h 37m</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>7.62</v>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>Official Duty</t>
         </is>
       </c>
-      <c r="H18" s="13" t="inlineStr">
-        <is>
-          <t>✈️ Live Airport Ground Station Duty (Logged in 08:00 AM / Awaiting Checkout | Free Zone Bus: Arr 07:03 PM, Dep 07:23 PM)</t>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>✈️ Live Daily Duty (Logged in 08:00 AM / Logged out 03:37 PM | Free Zone Bus: Arr 07:03 PM, Dep 07:23 PM)</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="14" t="inlineStr">
+      <c r="A20" s="11" t="inlineStr">
         <is>
           <t>Total October 2026 Hours</t>
         </is>
       </c>
-      <c r="F20" s="15">
+      <c r="F20" s="12">
         <f>SUM(F2:F18)</f>
         <v/>
       </c>
@@ -1647,12 +1632,12 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="14" t="inlineStr">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>Total September 2026 Hours</t>
         </is>
       </c>
-      <c r="F11" s="15">
+      <c r="F11" s="12">
         <f>SUM(F2:F9)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Update Oct 19 shift: Logged in at 07:55 AM (Official Duty)
</commit_message>
<xml_diff>
--- a/omar_elnemr_attendance_2026.xlsx
+++ b/omar_elnemr_attendance_2026.xlsx
@@ -44,7 +44,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -67,6 +67,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FCE4D6"/>
         <bgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -96,7 +102,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -126,6 +132,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -499,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1274,14 +1289,54 @@
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="11" t="inlineStr">
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>07:55 AM</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>To Be Updated</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F20" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="11" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="H20" s="13" t="inlineStr">
+        <is>
+          <t>✈️ Live Airport Ground Station Duty (Logged in 07:55 AM / Awaiting Checkout)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="14" t="inlineStr">
         <is>
           <t>Total October 2026 Hours</t>
         </is>
       </c>
-      <c r="F21" s="12">
-        <f>SUM(F2:F19)</f>
+      <c r="F22" s="15">
+        <f>SUM(F2:F20)</f>
         <v/>
       </c>
     </row>
@@ -1672,12 +1727,12 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="inlineStr">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>Total September 2026 Hours</t>
         </is>
       </c>
-      <c r="F11" s="12">
+      <c r="F11" s="15">
         <f>SUM(F2:F9)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Complete Oct 19 shift: Logged out at 03:20 PM (7h 25m)
</commit_message>
<xml_diff>
--- a/omar_elnemr_attendance_2026.xlsx
+++ b/omar_elnemr_attendance_2026.xlsx
@@ -44,7 +44,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -67,12 +67,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FCE4D6"/>
         <bgColor rgb="00FCE4D6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
-        <bgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -102,7 +96,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -132,15 +126,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1290,52 +1275,52 @@
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="11" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="B20" s="11" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>Monday</t>
         </is>
       </c>
-      <c r="C20" s="11" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>07:55 AM</t>
         </is>
       </c>
-      <c r="D20" s="11" t="inlineStr">
-        <is>
-          <t>To Be Updated</t>
-        </is>
-      </c>
-      <c r="E20" s="11" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="F20" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G20" s="11" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>03:20 PM</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>7h 25m</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>7.42</v>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>Official Duty</t>
         </is>
       </c>
-      <c r="H20" s="13" t="inlineStr">
-        <is>
-          <t>✈️ Live Airport Ground Station Duty (Logged in 07:55 AM / Awaiting Checkout)</t>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>✈️ Live Daily Duty (Logged in 07:55 AM / Logged out 03:20 PM)</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="14" t="inlineStr">
+      <c r="A22" s="11" t="inlineStr">
         <is>
           <t>Total October 2026 Hours</t>
         </is>
       </c>
-      <c r="F22" s="15">
+      <c r="F22" s="12">
         <f>SUM(F2:F20)</f>
         <v/>
       </c>
@@ -1727,12 +1712,12 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="14" t="inlineStr">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>Total September 2026 Hours</t>
         </is>
       </c>
-      <c r="F11" s="15">
+      <c r="F11" s="12">
         <f>SUM(F2:F9)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Update Oct 3-4 to 9.0h Paid Administrative Standby (airport pass delay)
</commit_message>
<xml_diff>
--- a/omar_elnemr_attendance_2026.xlsx
+++ b/omar_elnemr_attendance_2026.xlsx
@@ -647,7 +647,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>07:00 AM</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -657,20 +657,20 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>8h 00m</t>
+          <t>9h 00m</t>
         </is>
       </c>
       <c r="F4" s="3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Training / Paid</t>
+          <t>Paid Standby</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>🎓 Etihad IGS Training Prep / Paid Administrative Standby (8h)</t>
+          <t>🏢 Paid Administrative Standby (Damascus Airport Pass Delay - Company Paid)</t>
         </is>
       </c>
     </row>
@@ -687,7 +687,7 @@
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>07:45 AM</t>
+          <t>07:00 AM</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
@@ -697,20 +697,20 @@
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>8h 15m</t>
+          <t>9h 00m</t>
         </is>
       </c>
       <c r="F5" s="9" t="n">
-        <v>8.25</v>
+        <v>9</v>
       </c>
       <c r="G5" s="8" t="inlineStr">
         <is>
-          <t>Paid Shift</t>
+          <t>Paid Standby</t>
         </is>
       </c>
       <c r="H5" s="10" t="inlineStr">
         <is>
-          <t>🏢 Airport Onboarding Shift / Logged in 07:45 AM (8h 15m)</t>
+          <t>🏢 Paid Administrative Standby (Damascus Airport Pass Delay - Company Paid)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Oct 20 shift: Logged in at 07:55 AM (Official Duty)
</commit_message>
<xml_diff>
--- a/omar_elnemr_attendance_2026.xlsx
+++ b/omar_elnemr_attendance_2026.xlsx
@@ -44,7 +44,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -67,6 +67,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FCE4D6"/>
         <bgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -96,7 +102,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -126,6 +132,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -499,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1314,14 +1329,54 @@
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="11" t="inlineStr">
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="inlineStr">
+        <is>
+          <t>07:55 AM</t>
+        </is>
+      </c>
+      <c r="D21" s="11" t="inlineStr">
+        <is>
+          <t>To Be Updated</t>
+        </is>
+      </c>
+      <c r="E21" s="11" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F21" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="11" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="H21" s="13" t="inlineStr">
+        <is>
+          <t>✈️ Live Airport Ground Station Duty (Logged in 07:55 AM / Awaiting Checkout)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="14" t="inlineStr">
         <is>
           <t>Total October 2026 Hours</t>
         </is>
       </c>
-      <c r="F22" s="12">
-        <f>SUM(F2:F20)</f>
+      <c r="F23" s="15">
+        <f>SUM(F2:F21)</f>
         <v/>
       </c>
     </row>
@@ -1712,12 +1767,12 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="inlineStr">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>Total September 2026 Hours</t>
         </is>
       </c>
-      <c r="F11" s="12">
+      <c r="F11" s="15">
         <f>SUM(F2:F9)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Complete Oct 20 shift: Logged out at 06:24 PM (10h 29m / Overtime)
</commit_message>
<xml_diff>
--- a/omar_elnemr_attendance_2026.xlsx
+++ b/omar_elnemr_attendance_2026.xlsx
@@ -44,7 +44,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -67,12 +67,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FCE4D6"/>
         <bgColor rgb="00FCE4D6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
-        <bgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -102,7 +96,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -132,15 +126,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1330,52 +1315,52 @@
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="11" t="inlineStr">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>2026-10-20</t>
         </is>
       </c>
-      <c r="B21" s="11" t="inlineStr">
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t>Tuesday</t>
         </is>
       </c>
-      <c r="C21" s="11" t="inlineStr">
+      <c r="C21" s="8" t="inlineStr">
         <is>
           <t>07:55 AM</t>
         </is>
       </c>
-      <c r="D21" s="11" t="inlineStr">
-        <is>
-          <t>To Be Updated</t>
-        </is>
-      </c>
-      <c r="E21" s="11" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="F21" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G21" s="11" t="inlineStr">
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>06:24 PM</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>10h 29m</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="n">
+        <v>10.48</v>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
         <is>
           <t>Official Duty</t>
         </is>
       </c>
-      <c r="H21" s="13" t="inlineStr">
-        <is>
-          <t>✈️ Live Airport Ground Station Duty (Logged in 07:55 AM / Awaiting Checkout)</t>
+      <c r="H21" s="10" t="inlineStr">
+        <is>
+          <t>⚡ Extended Shift / Overtime (Logged in 07:55 AM / Logged out 06:24 PM)</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="14" t="inlineStr">
+      <c r="A23" s="11" t="inlineStr">
         <is>
           <t>Total October 2026 Hours</t>
         </is>
       </c>
-      <c r="F23" s="15">
+      <c r="F23" s="12">
         <f>SUM(F2:F21)</f>
         <v/>
       </c>
@@ -1767,12 +1752,12 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="14" t="inlineStr">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>Total September 2026 Hours</t>
         </is>
       </c>
-      <c r="F11" s="15">
+      <c r="F11" s="12">
         <f>SUM(F2:F9)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Update Omar Oct 23 shift: Logged in at 07:20 AM (Official Duty)
</commit_message>
<xml_diff>
--- a/omar_elnemr_attendance_2026.xlsx
+++ b/omar_elnemr_attendance_2026.xlsx
@@ -44,7 +44,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -67,6 +67,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FCE4D6"/>
         <bgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -96,7 +102,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -126,6 +132,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -499,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1434,14 +1449,54 @@
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="11" t="inlineStr">
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>07:20 AM</t>
+        </is>
+      </c>
+      <c r="D24" s="11" t="inlineStr">
+        <is>
+          <t>To Be Updated</t>
+        </is>
+      </c>
+      <c r="E24" s="11" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F24" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="11" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="H24" s="13" t="inlineStr">
+        <is>
+          <t>✈️ Live Daily Ground Duty (Logged in 07:20 AM / Awaiting Checkout)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="14" t="inlineStr">
         <is>
           <t>Total October 2026 Hours</t>
         </is>
       </c>
-      <c r="F25" s="12">
-        <f>SUM(F2:F23)</f>
+      <c r="F26" s="15">
+        <f>SUM(F2:F24)</f>
         <v/>
       </c>
     </row>
@@ -1832,12 +1887,12 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="inlineStr">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>Total September 2026 Hours</t>
         </is>
       </c>
-      <c r="F11" s="12">
+      <c r="F11" s="15">
         <f>SUM(F2:F9)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Update Omar Oct 24 shift: Logged in at 07:24 AM (Official Duty)
</commit_message>
<xml_diff>
--- a/omar_elnemr_attendance_2026.xlsx
+++ b/omar_elnemr_attendance_2026.xlsx
@@ -44,7 +44,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -67,6 +67,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FCE4D6"/>
         <bgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -96,7 +102,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -126,6 +132,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -499,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1474,14 +1489,54 @@
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="11" t="inlineStr">
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="C25" s="11" t="inlineStr">
+        <is>
+          <t>07:24 AM</t>
+        </is>
+      </c>
+      <c r="D25" s="11" t="inlineStr">
+        <is>
+          <t>To Be Updated</t>
+        </is>
+      </c>
+      <c r="E25" s="11" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F25" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="11" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="H25" s="13" t="inlineStr">
+        <is>
+          <t>✈️ Live Daily Ground Duty (Logged in 07:24 AM / Awaiting Checkout)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="14" t="inlineStr">
         <is>
           <t>Total October 2026 Hours</t>
         </is>
       </c>
-      <c r="F26" s="12">
-        <f>SUM(F2:F24)</f>
+      <c r="F27" s="15">
+        <f>SUM(F2:F25)</f>
         <v/>
       </c>
     </row>
@@ -1872,12 +1927,12 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="inlineStr">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>Total September 2026 Hours</t>
         </is>
       </c>
-      <c r="F11" s="12">
+      <c r="F11" s="15">
         <f>SUM(F2:F9)</f>
         <v/>
       </c>

</xml_diff>